<commit_message>
Complete data preprocessing and cleaning component
</commit_message>
<xml_diff>
--- a/data_retrieval/files/PA_JCR_SSCI_ESCI.xlsx
+++ b/data_retrieval/files/PA_JCR_SSCI_ESCI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stulsbuac-my.sharepoint.com/personal/e411394_lsbu_ac_uk/Documents/database_pa/data_retrieval/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="11_5C00C9B2E4AB6BB8C89969EFA0E25A273E7456E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5937209-BF50-4896-879C-A8856F1A0620}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="11_5C00C9B2E4AB6BB8C89969EFA0E25A273E7456E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96CBE613-2A8E-444A-8202-6F96DF6C6331}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FulvioScognamiglio_JCR_Journal" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="451">
   <si>
     <t>Journal name</t>
   </si>
@@ -1371,6 +1371,9 @@
   </si>
   <si>
     <t>ADMPUB</t>
+  </si>
+  <si>
+    <t>id:s4210198237</t>
   </si>
 </sst>
 </file>
@@ -1449,7 +1452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1461,7 +1464,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1484,19 +1486,19 @@
       </fill>
     </dxf>
     <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="0" tint="-0.14999847407452621"/>
           <bgColor theme="0" tint="-0.14999847407452621"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1527,11 +1529,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{51A121AE-4598-438A-909F-643FEF5F5D2A}" name="Table3" displayName="Table3" ref="A1:B89" totalsRowShown="0" dataDxfId="0" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{51A121AE-4598-438A-909F-643FEF5F5D2A}" name="Table3" displayName="Table3" ref="A1:B89" totalsRowShown="0" dataDxfId="3" tableBorderDxfId="2">
   <autoFilter ref="A1:B89" xr:uid="{51A121AE-4598-438A-909F-643FEF5F5D2A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{9D66A002-3996-45F8-8DA5-96A6EE4E245E}" name="Internal_name" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{8B6352B3-2CF3-4ABA-894E-6BC3FBA12FD6}" name="OpenAlex_ID" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{9D66A002-3996-45F8-8DA5-96A6EE4E245E}" name="Internal_name" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{8B6352B3-2CF3-4ABA-894E-6BC3FBA12FD6}" name="OpenAlex_ID" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1826,16 +1828,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F91"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1855,7 +1857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1875,7 +1877,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1895,7 +1897,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1915,7 +1917,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -1935,7 +1937,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1955,7 +1957,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1975,7 +1977,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1995,7 +1997,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -2015,7 +2017,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -2035,7 +2037,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -2055,7 +2057,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>57</v>
       </c>
@@ -2075,7 +2077,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -2095,7 +2097,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -2115,7 +2117,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>71</v>
       </c>
@@ -2135,7 +2137,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -2155,7 +2157,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -2175,7 +2177,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>86</v>
       </c>
@@ -2195,7 +2197,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>91</v>
       </c>
@@ -2215,7 +2217,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -2235,7 +2237,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>101</v>
       </c>
@@ -2255,7 +2257,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>106</v>
       </c>
@@ -2275,7 +2277,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>111</v>
       </c>
@@ -2295,7 +2297,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>116</v>
       </c>
@@ -2315,7 +2317,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>121</v>
       </c>
@@ -2335,7 +2337,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>126</v>
       </c>
@@ -2355,7 +2357,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>131</v>
       </c>
@@ -2375,7 +2377,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>136</v>
       </c>
@@ -2395,7 +2397,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>141</v>
       </c>
@@ -2415,7 +2417,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>146</v>
       </c>
@@ -2435,7 +2437,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>151</v>
       </c>
@@ -2455,7 +2457,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>156</v>
       </c>
@@ -2475,7 +2477,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>161</v>
       </c>
@@ -2495,7 +2497,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>166</v>
       </c>
@@ -2515,7 +2517,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>171</v>
       </c>
@@ -2535,7 +2537,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>176</v>
       </c>
@@ -2555,7 +2557,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>181</v>
       </c>
@@ -2575,7 +2577,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>186</v>
       </c>
@@ -2595,7 +2597,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>191</v>
       </c>
@@ -2615,7 +2617,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>196</v>
       </c>
@@ -2635,7 +2637,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>201</v>
       </c>
@@ -2655,7 +2657,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>206</v>
       </c>
@@ -2675,7 +2677,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>211</v>
       </c>
@@ -2695,7 +2697,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>216</v>
       </c>
@@ -2715,7 +2717,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>221</v>
       </c>
@@ -2735,7 +2737,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>226</v>
       </c>
@@ -2755,7 +2757,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>231</v>
       </c>
@@ -2775,7 +2777,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>236</v>
       </c>
@@ -2795,7 +2797,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>241</v>
       </c>
@@ -2815,7 +2817,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>246</v>
       </c>
@@ -2835,7 +2837,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>251</v>
       </c>
@@ -2855,7 +2857,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>255</v>
       </c>
@@ -2875,7 +2877,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>259</v>
       </c>
@@ -2895,7 +2897,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>262</v>
       </c>
@@ -2909,13 +2911,13 @@
         <v>249</v>
       </c>
       <c r="E54" t="s">
-        <v>159</v>
+        <v>450</v>
       </c>
       <c r="F54" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>264</v>
       </c>
@@ -2935,7 +2937,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>267</v>
       </c>
@@ -2955,7 +2957,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>271</v>
       </c>
@@ -2975,7 +2977,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>275</v>
       </c>
@@ -2995,7 +2997,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>279</v>
       </c>
@@ -3015,7 +3017,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>283</v>
       </c>
@@ -3035,7 +3037,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>287</v>
       </c>
@@ -3055,7 +3057,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>291</v>
       </c>
@@ -3075,7 +3077,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>295</v>
       </c>
@@ -3095,7 +3097,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>299</v>
       </c>
@@ -3115,7 +3117,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>303</v>
       </c>
@@ -3135,7 +3137,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>307</v>
       </c>
@@ -3155,7 +3157,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>311</v>
       </c>
@@ -3175,7 +3177,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>315</v>
       </c>
@@ -3195,7 +3197,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>319</v>
       </c>
@@ -3215,7 +3217,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>323</v>
       </c>
@@ -3235,7 +3237,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>327</v>
       </c>
@@ -3255,7 +3257,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>331</v>
       </c>
@@ -3275,7 +3277,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>335</v>
       </c>
@@ -3295,7 +3297,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>339</v>
       </c>
@@ -3315,7 +3317,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>343</v>
       </c>
@@ -3335,7 +3337,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>347</v>
       </c>
@@ -3355,7 +3357,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>351</v>
       </c>
@@ -3375,7 +3377,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>355</v>
       </c>
@@ -3395,7 +3397,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>359</v>
       </c>
@@ -3415,7 +3417,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>363</v>
       </c>
@@ -3435,7 +3437,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>367</v>
       </c>
@@ -3452,7 +3454,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>371</v>
       </c>
@@ -3472,7 +3474,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>375</v>
       </c>
@@ -3492,7 +3494,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>379</v>
       </c>
@@ -3512,7 +3514,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>383</v>
       </c>
@@ -3532,7 +3534,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>387</v>
       </c>
@@ -3552,7 +3554,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>391</v>
       </c>
@@ -3569,7 +3571,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>394</v>
       </c>
@@ -3589,7 +3591,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>398</v>
       </c>
@@ -3609,7 +3611,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>402</v>
       </c>
@@ -3629,7 +3631,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>406</v>
       </c>
@@ -3660,13 +3662,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{326D0DDD-3F26-41AD-A678-181630F98F54}">
   <dimension ref="A1:B89"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="1" max="1" width="16.1796875" customWidth="1"/>
+    <col min="2" max="2" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3674,7 +3676,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
@@ -3682,7 +3684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3690,7 +3692,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
@@ -3698,7 +3700,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -3706,7 +3708,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>31</v>
       </c>
@@ -3714,7 +3716,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -3722,7 +3724,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
@@ -3730,7 +3732,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -3738,7 +3740,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>51</v>
       </c>
@@ -3746,7 +3748,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>56</v>
       </c>
@@ -3754,7 +3756,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>61</v>
       </c>
@@ -3762,7 +3764,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -3770,7 +3772,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
@@ -3778,7 +3780,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>75</v>
       </c>
@@ -3786,7 +3788,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>80</v>
       </c>
@@ -3794,7 +3796,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -3802,7 +3804,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>90</v>
       </c>
@@ -3810,7 +3812,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>95</v>
       </c>
@@ -3818,7 +3820,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>100</v>
       </c>
@@ -3826,7 +3828,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>105</v>
       </c>
@@ -3834,7 +3836,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>110</v>
       </c>
@@ -3842,7 +3844,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>115</v>
       </c>
@@ -3850,7 +3852,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>120</v>
       </c>
@@ -3858,7 +3860,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>125</v>
       </c>
@@ -3866,7 +3868,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>130</v>
       </c>
@@ -3874,7 +3876,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>135</v>
       </c>
@@ -3882,7 +3884,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>140</v>
       </c>
@@ -3890,7 +3892,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>145</v>
       </c>
@@ -3898,7 +3900,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>150</v>
       </c>
@@ -3906,7 +3908,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>155</v>
       </c>
@@ -3914,7 +3916,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>160</v>
       </c>
@@ -3922,7 +3924,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>165</v>
       </c>
@@ -3930,7 +3932,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>170</v>
       </c>
@@ -3938,7 +3940,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>175</v>
       </c>
@@ -3946,7 +3948,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>180</v>
       </c>
@@ -3954,7 +3956,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>185</v>
       </c>
@@ -3962,7 +3964,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>190</v>
       </c>
@@ -3970,7 +3972,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>195</v>
       </c>
@@ -3978,7 +3980,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>200</v>
       </c>
@@ -3986,7 +3988,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>205</v>
       </c>
@@ -3994,7 +3996,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>210</v>
       </c>
@@ -4002,7 +4004,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>215</v>
       </c>
@@ -4010,7 +4012,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>220</v>
       </c>
@@ -4018,7 +4020,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>225</v>
       </c>
@@ -4026,7 +4028,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>230</v>
       </c>
@@ -4034,7 +4036,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>235</v>
       </c>
@@ -4042,7 +4044,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>240</v>
       </c>
@@ -4050,7 +4052,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>245</v>
       </c>
@@ -4058,7 +4060,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>410</v>
       </c>
@@ -4066,7 +4068,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>411</v>
       </c>
@@ -4074,7 +4076,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
         <v>416</v>
       </c>
@@ -4082,7 +4084,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>417</v>
       </c>
@@ -4090,15 +4092,15 @@
         <v>261</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>414</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>418</v>
       </c>
@@ -4106,7 +4108,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>419</v>
       </c>
@@ -4114,7 +4116,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>420</v>
       </c>
@@ -4122,7 +4124,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>421</v>
       </c>
@@ -4130,7 +4132,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>422</v>
       </c>
@@ -4138,7 +4140,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>423</v>
       </c>
@@ -4146,7 +4148,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>424</v>
       </c>
@@ -4154,7 +4156,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>415</v>
       </c>
@@ -4162,7 +4164,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>425</v>
       </c>
@@ -4170,7 +4172,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>412</v>
       </c>
@@ -4178,7 +4180,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>426</v>
       </c>
@@ -4186,7 +4188,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
         <v>427</v>
       </c>
@@ -4194,7 +4196,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>428</v>
       </c>
@@ -4202,7 +4204,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
         <v>429</v>
       </c>
@@ -4210,7 +4212,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>430</v>
       </c>
@@ -4218,7 +4220,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
         <v>432</v>
       </c>
@@ -4226,7 +4228,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>431</v>
       </c>
@@ -4234,7 +4236,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>436</v>
       </c>
@@ -4242,7 +4244,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>437</v>
       </c>
@@ -4250,7 +4252,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>438</v>
       </c>
@@ -4258,7 +4260,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>433</v>
       </c>
@@ -4266,7 +4268,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
         <v>439</v>
       </c>
@@ -4274,7 +4276,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>440</v>
       </c>
@@ -4282,7 +4284,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
         <v>441</v>
       </c>
@@ -4290,7 +4292,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>442</v>
       </c>
@@ -4298,7 +4300,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>443</v>
       </c>
@@ -4306,7 +4308,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
         <v>444</v>
       </c>
@@ -4314,7 +4316,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>445</v>
       </c>
@@ -4322,7 +4324,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
         <v>434</v>
       </c>
@@ -4330,7 +4332,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>435</v>
       </c>
@@ -4338,7 +4340,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
         <v>446</v>
       </c>
@@ -4346,7 +4348,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
         <v>447</v>
       </c>
@@ -4354,7 +4356,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>448</v>
       </c>
@@ -4362,7 +4364,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
         <v>413</v>
       </c>
@@ -4370,18 +4372,19 @@
         <v>405</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="5" t="s">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>449</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="B89" t="s">
         <v>409</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>